<commit_message>
Pipeline rules, C26100 completion, and office workspace sync.
Add shipment-pipeline-order and session-turn-closeout rules; align handoff and preflight. Ship C26089-C26100 metadata, gate reports, ship-stats bundle, scripts, and web pipeline.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/1_Input_Raw/Shipments/EF-C26079-C04-36460  桌布-2026.7.10/出货表/C04-2616-U-2026.7.31.xlsx
+++ b/1_Input_Raw/Shipments/EF-C26079-C04-36460  桌布-2026.7.10/出货表/C04-2616-U-2026.7.31.xlsx
@@ -752,7 +752,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -866,6 +866,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1256,7 +1265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="18.25" customWidth="1" style="35" min="1" max="1"/>
@@ -1379,7 +1388,7 @@
           <t>平纹单面磨毛桌布</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
+      <c r="B5" s="39" t="inlineStr">
         <is>
           <t>90克/平方米</t>
         </is>
@@ -1397,18 +1406,22 @@
       <c r="E5" s="15" t="n">
         <v>2000</v>
       </c>
-      <c r="F5" s="39" t="n"/>
-      <c r="G5" s="21" t="n"/>
-      <c r="H5" s="22" t="n"/>
-      <c r="I5" s="17" t="inlineStr">
+      <c r="F5" s="40" t="inlineStr">
+        <is>
+          <t>C26079</t>
+        </is>
+      </c>
+      <c r="G5" s="37" t="n"/>
+      <c r="H5" s="37" t="n"/>
+      <c r="I5" s="41" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
     </row>
     <row r="6" ht="37" customHeight="1" s="35">
-      <c r="A6" s="39" t="n"/>
-      <c r="B6" s="39" t="n"/>
+      <c r="A6" s="42" t="n"/>
+      <c r="B6" s="42" t="n"/>
       <c r="C6" s="14" t="inlineStr">
         <is>
           <t>60X102inch</t>
@@ -1422,14 +1435,14 @@
       <c r="E6" s="15" t="n">
         <v>2280</v>
       </c>
-      <c r="F6" s="39" t="n"/>
-      <c r="G6" s="21" t="n"/>
-      <c r="H6" s="22" t="n"/>
-      <c r="I6" s="39" t="n"/>
+      <c r="F6" s="42" t="n"/>
+      <c r="G6" s="37" t="n"/>
+      <c r="H6" s="37" t="n"/>
+      <c r="I6" s="42" t="n"/>
     </row>
     <row r="7" ht="37" customHeight="1" s="35">
-      <c r="A7" s="39" t="n"/>
-      <c r="B7" s="39" t="n"/>
+      <c r="A7" s="42" t="n"/>
+      <c r="B7" s="42" t="n"/>
       <c r="C7" s="14" t="inlineStr">
         <is>
           <t>60X102inch</t>
@@ -1443,14 +1456,14 @@
       <c r="E7" s="15" t="n">
         <v>10480</v>
       </c>
-      <c r="F7" s="39" t="n"/>
-      <c r="G7" s="21" t="n"/>
-      <c r="H7" s="22" t="n"/>
-      <c r="I7" s="39" t="n"/>
+      <c r="F7" s="42" t="n"/>
+      <c r="G7" s="37" t="n"/>
+      <c r="H7" s="37" t="n"/>
+      <c r="I7" s="42" t="n"/>
     </row>
     <row r="8" ht="37" customHeight="1" s="35">
-      <c r="A8" s="39" t="n"/>
-      <c r="B8" s="39" t="n"/>
+      <c r="A8" s="42" t="n"/>
+      <c r="B8" s="42" t="n"/>
       <c r="C8" s="14" t="inlineStr">
         <is>
           <t>60X126inch</t>
@@ -1464,14 +1477,14 @@
       <c r="E8" s="15" t="n">
         <v>3660</v>
       </c>
-      <c r="F8" s="39" t="n"/>
-      <c r="G8" s="21" t="n"/>
-      <c r="H8" s="22" t="n"/>
-      <c r="I8" s="39" t="n"/>
+      <c r="F8" s="42" t="n"/>
+      <c r="G8" s="37" t="n"/>
+      <c r="H8" s="37" t="n"/>
+      <c r="I8" s="42" t="n"/>
     </row>
     <row r="9" ht="37" customHeight="1" s="35">
-      <c r="A9" s="39" t="n"/>
-      <c r="B9" s="39" t="n"/>
+      <c r="A9" s="42" t="n"/>
+      <c r="B9" s="42" t="n"/>
       <c r="C9" s="14" t="inlineStr">
         <is>
           <t>60X126inch</t>
@@ -1485,14 +1498,14 @@
       <c r="E9" s="15" t="n">
         <v>2280</v>
       </c>
-      <c r="F9" s="39" t="n"/>
-      <c r="G9" s="21" t="n"/>
-      <c r="H9" s="22" t="n"/>
-      <c r="I9" s="39" t="n"/>
+      <c r="F9" s="42" t="n"/>
+      <c r="G9" s="37" t="n"/>
+      <c r="H9" s="37" t="n"/>
+      <c r="I9" s="42" t="n"/>
     </row>
     <row r="10" ht="37" customHeight="1" s="35">
-      <c r="A10" s="39" t="n"/>
-      <c r="B10" s="39" t="n"/>
+      <c r="A10" s="42" t="n"/>
+      <c r="B10" s="42" t="n"/>
       <c r="C10" s="14" t="inlineStr">
         <is>
           <t>70X120inch</t>
@@ -1506,14 +1519,14 @@
       <c r="E10" s="15" t="n">
         <v>3300</v>
       </c>
-      <c r="F10" s="39" t="n"/>
-      <c r="G10" s="21" t="n"/>
-      <c r="H10" s="22" t="n"/>
-      <c r="I10" s="39" t="n"/>
+      <c r="F10" s="42" t="n"/>
+      <c r="G10" s="37" t="n"/>
+      <c r="H10" s="37" t="n"/>
+      <c r="I10" s="42" t="n"/>
     </row>
     <row r="11" ht="37" customHeight="1" s="35">
-      <c r="A11" s="39" t="n"/>
-      <c r="B11" s="39" t="n"/>
+      <c r="A11" s="42" t="n"/>
+      <c r="B11" s="42" t="n"/>
       <c r="C11" s="14" t="inlineStr">
         <is>
           <t>70X120inch</t>
@@ -1527,14 +1540,14 @@
       <c r="E11" s="15" t="n">
         <v>3000</v>
       </c>
-      <c r="F11" s="39" t="n"/>
-      <c r="G11" s="21" t="n"/>
-      <c r="H11" s="22" t="n"/>
-      <c r="I11" s="39" t="n"/>
+      <c r="F11" s="42" t="n"/>
+      <c r="G11" s="37" t="n"/>
+      <c r="H11" s="37" t="n"/>
+      <c r="I11" s="42" t="n"/>
     </row>
     <row r="12" ht="37" customHeight="1" s="35">
-      <c r="A12" s="39" t="n"/>
-      <c r="B12" s="39" t="n"/>
+      <c r="A12" s="42" t="n"/>
+      <c r="B12" s="42" t="n"/>
       <c r="C12" s="14" t="inlineStr">
         <is>
           <t>70X120inch</t>
@@ -1548,14 +1561,14 @@
       <c r="E12" s="15" t="n">
         <v>600</v>
       </c>
-      <c r="F12" s="39" t="n"/>
-      <c r="G12" s="21" t="n"/>
-      <c r="H12" s="22" t="n"/>
-      <c r="I12" s="39" t="n"/>
+      <c r="F12" s="42" t="n"/>
+      <c r="G12" s="37" t="n"/>
+      <c r="H12" s="37" t="n"/>
+      <c r="I12" s="42" t="n"/>
     </row>
     <row r="13" ht="37" customHeight="1" s="35">
-      <c r="A13" s="39" t="n"/>
-      <c r="B13" s="39" t="n"/>
+      <c r="A13" s="42" t="n"/>
+      <c r="B13" s="42" t="n"/>
       <c r="C13" s="14" t="inlineStr">
         <is>
           <t>90 inch round</t>
@@ -1569,14 +1582,14 @@
       <c r="E13" s="15" t="n">
         <v>5760</v>
       </c>
-      <c r="F13" s="39" t="n"/>
-      <c r="G13" s="21" t="n"/>
-      <c r="H13" s="22" t="n"/>
-      <c r="I13" s="39" t="n"/>
+      <c r="F13" s="42" t="n"/>
+      <c r="G13" s="37" t="n"/>
+      <c r="H13" s="37" t="n"/>
+      <c r="I13" s="42" t="n"/>
     </row>
     <row r="14" ht="37" customHeight="1" s="35">
-      <c r="A14" s="39" t="n"/>
-      <c r="B14" s="39" t="n"/>
+      <c r="A14" s="42" t="n"/>
+      <c r="B14" s="42" t="n"/>
       <c r="C14" s="14" t="inlineStr">
         <is>
           <t>90 inch round</t>
@@ -1590,14 +1603,14 @@
       <c r="E14" s="15" t="n">
         <v>2100</v>
       </c>
-      <c r="F14" s="39" t="n"/>
-      <c r="G14" s="21" t="n"/>
-      <c r="H14" s="22" t="n"/>
-      <c r="I14" s="39" t="n"/>
+      <c r="F14" s="42" t="n"/>
+      <c r="G14" s="37" t="n"/>
+      <c r="H14" s="37" t="n"/>
+      <c r="I14" s="42" t="n"/>
     </row>
     <row r="15" ht="37" customHeight="1" s="35">
-      <c r="A15" s="40" t="n"/>
-      <c r="B15" s="40" t="n"/>
+      <c r="A15" s="43" t="n"/>
+      <c r="B15" s="43" t="n"/>
       <c r="C15" s="14" t="inlineStr">
         <is>
           <t>90 inch round</t>
@@ -1611,52 +1624,51 @@
       <c r="E15" s="15" t="n">
         <v>1000</v>
       </c>
-      <c r="F15" s="39" t="n"/>
-      <c r="G15" s="21" t="n"/>
-      <c r="H15" s="22" t="n"/>
-      <c r="I15" s="39" t="n"/>
+      <c r="F15" s="43" t="n"/>
+      <c r="G15" s="37" t="n"/>
+      <c r="H15" s="37" t="n"/>
+      <c r="I15" s="42" t="n"/>
     </row>
     <row r="16" ht="37" customHeight="1" s="35">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="38" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B16" s="27" t="n"/>
-      <c r="C16" s="27" t="n"/>
-      <c r="D16" s="27" t="n"/>
-      <c r="E16" s="28">
+      <c r="B16" s="22" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="14" t="n"/>
+      <c r="E16" s="15">
         <f>SUM(E5:E15)</f>
         <v/>
       </c>
-      <c r="F16" s="21" t="n"/>
-      <c r="G16" s="21" t="n"/>
-      <c r="H16" s="22" t="n"/>
-      <c r="I16" s="29" t="n"/>
+      <c r="F16" s="15" t="n"/>
+      <c r="G16" s="37" t="n"/>
+      <c r="H16" s="37" t="n"/>
+      <c r="I16" s="17" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="39" t="n"/>
-      <c r="B17" s="39" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="14" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="39" t="n"/>
-      <c r="G17" s="21" t="n"/>
-      <c r="H17" s="22" t="n"/>
-      <c r="I17" s="39" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="39" t="n"/>
-      <c r="B18" s="39" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="14" t="n"/>
-      <c r="E18" s="15" t="n"/>
-      <c r="F18" s="39" t="n"/>
-      <c r="G18" s="21" t="n"/>
-      <c r="H18" s="22" t="n"/>
-      <c r="I18" s="39" t="n"/>
-      <c r="J18" s="34" t="n"/>
-    </row>
+      <c r="A17" s="30" t="n"/>
+      <c r="B17" s="30" t="n"/>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="31" t="n"/>
+      <c r="E17" s="31" t="n"/>
+      <c r="F17" s="32" t="n"/>
+      <c r="G17" s="32" t="n"/>
+      <c r="H17" s="33" t="n"/>
+    </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20">
+      <c r="J20" s="34" t="n"/>
+    </row>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="F5:F15"/>

</xml_diff>